<commit_message>
New Backstop technology & PRK SAM
- TSF
- PRK SAM
</commit_message>
<xml_diff>
--- a/3.SAM/Input_CGE/Backstop_Technology.xlsx
+++ b/3.SAM/Input_CGE/Backstop_Technology.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kimc0\GUIDE_GLOBAL_CGE\2.RD_CGE\Input_w-t\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kimc0\GUIDE_GLOBAL_CGE\2.RD_CGE\Input_CGE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6500863-5DF4-48A7-8137-185D77F75C67}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF2A024-68A7-434D-BD2A-C70DB18D3FEF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Capital" sheetId="1" r:id="rId1"/>
     <sheet name="Labor" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -176,6 +176,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -240,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -251,6 +254,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -1168,55 +1173,55 @@
       <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="7">
         <v>0.13766860208102766</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="7">
         <v>8.6109773345080784E-2</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="7">
         <v>0.10161828258689634</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="7">
         <v>8.3572234945448534E-2</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="7">
         <v>1.6261972049879031E-2</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="7">
         <v>0.30256765387797679</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="7">
         <v>0.17025571296755587</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="7">
         <v>0.12494498037552584</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="7">
         <v>0.13711238635885875</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="7">
         <v>0.12557425449537674</v>
       </c>
-      <c r="L12" s="1">
+      <c r="L12" s="7">
         <v>0.11495754797625871</v>
       </c>
-      <c r="M12" s="1">
+      <c r="M12" s="7">
         <v>0.2592554126317072</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="7">
         <v>0.15359873816344011</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="7">
         <v>4.7097319852229411E-2</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="7">
         <v>0.12756239125630367</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="7">
         <v>0.13390264487803155</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="7">
         <v>0.11626092883199282</v>
       </c>
     </row>
@@ -1224,55 +1229,55 @@
       <c r="A13" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="7">
         <v>0.25579691625407447</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="7">
         <v>0.20999971281131649</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="7">
         <v>0.32143085894709383</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="7">
         <v>0.15311102528916365</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="7">
         <v>0.15114048435940483</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="7">
         <v>0.41140981458373665</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="7">
         <v>0.23294697963716798</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="7">
         <v>0.24379222432454484</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="7">
         <v>0.18225444595797535</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="7">
         <v>0.23199563759326919</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="7">
         <v>0.23968552953058264</v>
       </c>
-      <c r="M13" s="1">
+      <c r="M13" s="7">
         <v>0.52859719820720907</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="7">
         <v>0.34247914736639462</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="7">
         <v>0.11746714236577584</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="7">
         <v>0.27983097544002478</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="7">
         <v>0.25066375281357012</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="7">
         <v>0.19995753938182728</v>
       </c>
     </row>
@@ -1280,55 +1285,55 @@
       <c r="A14" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="7">
         <v>0.11172030629930593</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="7">
         <v>0.10503551443483379</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="7">
         <v>0.11039457350102014</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="7">
         <v>0.12450520660576016</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="7">
         <v>4.3819736641679548E-2</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="7">
         <v>0.46796704513335413</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="7">
         <v>0.1050281071295963</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="7">
         <v>0.13175575333659997</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="7">
         <v>6.5984254191029573E-2</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="7">
         <v>8.1812913353796951E-2</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="7">
         <v>0.10376359144158755</v>
       </c>
-      <c r="M14" s="1">
+      <c r="M14" s="7">
         <v>0.34190199212123329</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="7">
         <v>7.1140906111524974E-2</v>
       </c>
-      <c r="O14" s="1">
+      <c r="O14" s="7">
         <v>6.9156149444488973E-2</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="7">
         <v>5.3147237867405203E-2</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="7">
         <v>9.6315994869283078E-2</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="7">
         <v>5.7291108308303682E-2</v>
       </c>
     </row>
@@ -2120,55 +2125,55 @@
       <c r="A29" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="7">
         <v>0.25433159797660349</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="7">
         <v>0.38658505185768749</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="7">
         <v>0.34120691306584811</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="7">
         <v>0.38068135945167619</v>
       </c>
-      <c r="F29" s="1">
+      <c r="F29" s="7">
         <v>0.35122140751409198</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29" s="7">
         <v>0.11281970375175594</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="7">
         <v>0.21127736933949604</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29" s="7">
         <v>0.35630493671993169</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="7">
         <v>0.19288400250979254</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="7">
         <v>0.1474333349882101</v>
       </c>
-      <c r="L29" s="1">
+      <c r="L29" s="7">
         <v>0.39838226416109335</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="7">
         <v>0.4881137468592327</v>
       </c>
-      <c r="N29" s="1">
+      <c r="N29" s="7">
         <v>0.32323517361713539</v>
       </c>
-      <c r="O29" s="1">
+      <c r="O29" s="7">
         <v>0.14019801518934541</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="7">
         <v>0.35565807370142632</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="7">
         <v>0.43644983218240352</v>
       </c>
-      <c r="R29" s="1">
+      <c r="R29" s="7">
         <v>0.30330665574738708</v>
       </c>
     </row>
@@ -2176,55 +2181,55 @@
       <c r="A30" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="7">
         <v>0.1170736715064392</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="7">
         <v>0.15110492405396198</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="7">
         <v>0.13205907037968057</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="7">
         <v>0.13895387653750038</v>
       </c>
-      <c r="F30" s="1">
+      <c r="F30" s="7">
         <v>0.12148761767578416</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30" s="7">
         <v>7.3308226700085022E-2</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="7">
         <v>9.0190351062195431E-2</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30" s="7">
         <v>0.12003511518661149</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="7">
         <v>0.12150016117359913</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="7">
         <v>0.12486164058444817</v>
       </c>
-      <c r="L30" s="1">
+      <c r="L30" s="7">
         <v>0.15647449483146286</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="7">
         <v>0.14232105624304747</v>
       </c>
-      <c r="N30" s="1">
+      <c r="N30" s="7">
         <v>0.1043908750790072</v>
       </c>
-      <c r="O30" s="1">
+      <c r="O30" s="7">
         <v>5.7641513236838762E-2</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="7">
         <v>0.11400482639517379</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="7">
         <v>0.20446362108014191</v>
       </c>
-      <c r="R30" s="1">
+      <c r="R30" s="7">
         <v>0.17505303888672649</v>
       </c>
     </row>
@@ -2232,55 +2237,55 @@
       <c r="A31" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="7">
         <v>0.20486358181122283</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" s="7">
         <v>0.22901864381912251</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="7">
         <v>0.20639193281690757</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="7">
         <v>0.1504384203614858</v>
       </c>
-      <c r="F31" s="1">
+      <c r="F31" s="7">
         <v>0.251279268956135</v>
       </c>
-      <c r="G31" s="1">
+      <c r="G31" s="7">
         <v>9.5277910574936162E-2</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="7">
         <v>0.17464525872089784</v>
       </c>
-      <c r="I31" s="1">
+      <c r="I31" s="7">
         <v>0.19728262374114597</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="7">
         <v>9.4173838806997021E-2</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="7">
         <v>8.0338178518777489E-2</v>
       </c>
-      <c r="L31" s="1">
+      <c r="L31" s="7">
         <v>0.23591762325230931</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="7">
         <v>0.21903364093880603</v>
       </c>
-      <c r="N31" s="1">
+      <c r="N31" s="7">
         <v>0.18435411057847817</v>
       </c>
-      <c r="O31" s="1">
+      <c r="O31" s="7">
         <v>0.11856451154295786</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="7">
         <v>0.18167878727816222</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="7">
         <v>0.2159707334483266</v>
       </c>
-      <c r="R31" s="1">
+      <c r="R31" s="7">
         <v>8.991949308491598E-2</v>
       </c>
     </row>
@@ -2339,6 +2344,139 @@
       <c r="R32" s="1">
         <v>0</v>
       </c>
+    </row>
+    <row r="38" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6"/>
+      <c r="K38" s="6"/>
+      <c r="L38" s="6"/>
+      <c r="M38" s="6"/>
+      <c r="N38" s="6"/>
+      <c r="O38" s="6"/>
+      <c r="P38" s="6"/>
+      <c r="Q38" s="6"/>
+      <c r="R38" s="6"/>
+    </row>
+    <row r="39" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="6"/>
+      <c r="K39" s="6"/>
+      <c r="L39" s="6"/>
+      <c r="M39" s="6"/>
+      <c r="N39" s="6"/>
+      <c r="O39" s="6"/>
+      <c r="P39" s="6"/>
+      <c r="Q39" s="6"/>
+      <c r="R39" s="6"/>
+    </row>
+    <row r="40" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6"/>
+      <c r="K40" s="6"/>
+      <c r="L40" s="6"/>
+      <c r="M40" s="6"/>
+      <c r="N40" s="6"/>
+      <c r="O40" s="6"/>
+      <c r="P40" s="6"/>
+      <c r="Q40" s="6"/>
+      <c r="R40" s="6"/>
+    </row>
+    <row r="41" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="6"/>
+      <c r="L41" s="6"/>
+      <c r="M41" s="6"/>
+      <c r="N41" s="6"/>
+      <c r="O41" s="6"/>
+      <c r="P41" s="6"/>
+      <c r="Q41" s="6"/>
+      <c r="R41" s="6"/>
+    </row>
+    <row r="42" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6"/>
+      <c r="L42" s="6"/>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="6"/>
+      <c r="P42" s="6"/>
+      <c r="Q42" s="6"/>
+      <c r="R42" s="6"/>
+    </row>
+    <row r="43" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
+      <c r="R43" s="6"/>
+    </row>
+    <row r="44" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B44" s="6"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="6"/>
+      <c r="N44" s="6"/>
+      <c r="O44" s="6"/>
+      <c r="P44" s="6"/>
+      <c r="Q44" s="6"/>
+      <c r="R44" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2985,55 +3123,55 @@
       <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="7">
         <v>0.13744423314688914</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="7">
         <v>0.1311652537319537</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="7">
         <v>0.15679015469507329</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="7">
         <v>0.11269118973067596</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="7">
         <v>1.9801259295260283E-3</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="7">
         <v>0.77308838990921491</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="7">
         <v>0.1855799643631974</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="7">
         <v>0.20743013088094833</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="7">
         <v>0.20618903584151393</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="7">
         <v>0.15871549998929796</v>
       </c>
-      <c r="L12" s="1">
+      <c r="L12" s="7">
         <v>0.15761885982375581</v>
       </c>
-      <c r="M12" s="1">
+      <c r="M12" s="7">
         <v>0.17165553733030059</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="7">
         <v>0.19447039592305576</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="7">
         <v>0.10946801046118662</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="7">
         <v>0.12387747224263464</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="7">
         <v>0.12347183053158821</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="7">
         <v>0.31407310510517195</v>
       </c>
     </row>
@@ -3041,55 +3179,55 @@
       <c r="A13" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="7">
         <v>0.1058913706218628</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="7">
         <v>9.9484154898865473E-2</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="7">
         <v>0.15080523036838142</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="7">
         <v>0.12013933569413413</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="7">
         <v>7.4879144064073214E-2</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="7">
         <v>0.32210621294142894</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="7">
         <v>0.18623482938292801</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="7">
         <v>0.14767759415516671</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="7">
         <v>0.15343002912449899</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="7">
         <v>0.10752405539621313</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="7">
         <v>0.1018248984166166</v>
       </c>
-      <c r="M13" s="1">
+      <c r="M13" s="7">
         <v>0.15038221433415752</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="7">
         <v>9.8527517468661688E-2</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="7">
         <v>8.0626483972680144E-2</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="7">
         <v>7.7506251693013076E-2</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="7">
         <v>9.9948338954808369E-2</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="7">
         <v>0.16281235655455376</v>
       </c>
     </row>
@@ -3097,55 +3235,55 @@
       <c r="A14" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="7">
         <v>4.0290637136686111E-2</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="7">
         <v>3.6399241749338208E-2</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="7">
         <v>2.4064440934770698E-2</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="7">
         <v>2.521180873627013E-2</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="7">
         <v>1.2529361307975512E-3</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="7">
         <v>0.15991314517678659</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="7">
         <v>5.6357687145266615E-2</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="7">
         <v>4.3235345536590405E-2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="7">
         <v>5.5798579982420521E-2</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="7">
         <v>4.3647057786760347E-2</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="7">
         <v>3.7268541930229909E-2</v>
       </c>
-      <c r="M14" s="1">
+      <c r="M14" s="7">
         <v>3.094179890629515E-2</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="7">
         <v>2.7080035083535566E-2</v>
       </c>
-      <c r="O14" s="1">
+      <c r="O14" s="7">
         <v>3.6174760161615131E-2</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="7">
         <v>1.6527202710774055E-2</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="7">
         <v>3.2757410402628098E-2</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="7">
         <v>0.11057399789130432</v>
       </c>
     </row>
@@ -3937,55 +4075,55 @@
       <c r="A29" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="7">
         <v>0.22169357923814365</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="7">
         <v>0.16041144335575966</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="7">
         <v>0.22023913928338917</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="7">
         <v>0.13854904217598785</v>
       </c>
-      <c r="F29" s="1">
+      <c r="F29" s="7">
         <v>0.10557539846566108</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29" s="7">
         <v>5.5827837333378608E-2</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="7">
         <v>0.20906848854729287</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29" s="7">
         <v>0.20442325622779747</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="7">
         <v>0.17027179173780971</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="7">
         <v>0.12130713396690607</v>
       </c>
-      <c r="L29" s="1">
+      <c r="L29" s="7">
         <v>0.12759109220617895</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="7">
         <v>0.15260090312235289</v>
       </c>
-      <c r="N29" s="1">
+      <c r="N29" s="7">
         <v>0.20036751569593902</v>
       </c>
-      <c r="O29" s="1">
+      <c r="O29" s="7">
         <v>0.12019263927752655</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="7">
         <v>0.20987657799296955</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="7">
         <v>0.17410543637040221</v>
       </c>
-      <c r="R29" s="1">
+      <c r="R29" s="7">
         <v>0.19018049622827704</v>
       </c>
     </row>
@@ -3993,55 +4131,55 @@
       <c r="A30" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="7">
         <v>0.11458184420461842</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="7">
         <v>0.1692810977657177</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="7">
         <v>0.19538029013637431</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="7">
         <v>0.30147389186869922</v>
       </c>
-      <c r="F30" s="1">
+      <c r="F30" s="7">
         <v>4.6391012091991896E-2</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30" s="7">
         <v>7.160802200981245E-2</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="7">
         <v>0.16665925967851519</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30" s="7">
         <v>0.18995294096106996</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="7">
         <v>0.14326679637068843</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="7">
         <v>0.16330202362381288</v>
       </c>
-      <c r="L30" s="1">
+      <c r="L30" s="7">
         <v>0.2698916390862322</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="7">
         <v>0.20184339294642983</v>
       </c>
-      <c r="N30" s="1">
+      <c r="N30" s="7">
         <v>0.1480211159833002</v>
       </c>
-      <c r="O30" s="1">
+      <c r="O30" s="7">
         <v>0.23711527906136712</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="7">
         <v>0.28675624921121612</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="7">
         <v>0.16093049265001369</v>
       </c>
-      <c r="R30" s="1">
+      <c r="R30" s="7">
         <v>0.23897831783627196</v>
       </c>
     </row>
@@ -4049,55 +4187,55 @@
       <c r="A31" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="7">
         <v>0.12220255451789672</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" s="7">
         <v>0.12087428202833772</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="7">
         <v>8.3054559835810324E-2</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="7">
         <v>0.10743604596429031</v>
       </c>
-      <c r="F31" s="1">
+      <c r="F31" s="7">
         <v>8.3719641534616251E-2</v>
       </c>
-      <c r="G31" s="1">
+      <c r="G31" s="7">
         <v>3.141864158796577E-2</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="7">
         <v>0.18942916253553149</v>
       </c>
-      <c r="I31" s="1">
+      <c r="I31" s="7">
         <v>0.10944661484475124</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="7">
         <v>8.5760034112021544E-2</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="7">
         <v>0.10471524688439497</v>
       </c>
-      <c r="L31" s="1">
+      <c r="L31" s="7">
         <v>9.7460424476299656E-2</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="7">
         <v>0.1325536913659266</v>
       </c>
-      <c r="N31" s="1">
+      <c r="N31" s="7">
         <v>0.12451844137173253</v>
       </c>
-      <c r="O31" s="1">
+      <c r="O31" s="7">
         <v>0.17933651350515462</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="7">
         <v>0.13258095243895213</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="7">
         <v>0.12102045069158608</v>
       </c>
-      <c r="R31" s="1">
+      <c r="R31" s="7">
         <v>0.17552640179411408</v>
       </c>
     </row>

</xml_diff>